<commit_message>
Add multi-case suites and action-only locator self-healing
</commit_message>
<xml_diff>
--- a/cases/osm/WBS_testcase1_osm.xlsx
+++ b/cases/osm/WBS_testcase1_osm.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="23">
   <si>
     <t>TestCase_ID</t>
   </si>
@@ -53,15 +53,55 @@
 5. Observe or check the Estimated Arrival Time (ETA)  </t>
   </si>
   <si>
-    <t xml:space="preserve">1. OSM is open in browser
+    <t>1. OSM is open in browser
 2. The starting-point and destination fields are visible.
 3. Car/ Driving is selected
 4. The map correctly display the route from Hamburg to Berlin. 
-5. The displayed estimated driving journey duration is under 3 hours (strictly less than 180 minutes).
+5. The displayed estimated driving journey duration is under 3 hours (strictly less than 180 minutes).</t>
+  </si>
+  <si>
+    <t>Clean up all the input</t>
+  </si>
+  <si>
+    <t>OSM-002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open Street Map
+2. Click on Route Planning
+3. Select Car or driving
+4. Enter Hamburg as the starting point and Munich as the destination. Request directions to start the route search.
+5. Observe or check the Estimated Arrival Time (ETA)  </t>
+  </si>
+  <si>
+    <t>1. OSM is open in browser
+2. The starting-point and destination fields are visible.
+3. Car/ Driving is selected
+4. The map correctly display the route from Hamburg to Munich or München. 
+5. The displayed estimated driving journey duration is under 3 hours (strictly less than 180 minutes).</t>
+  </si>
+  <si>
+    <t>OSM-003</t>
+  </si>
+  <si>
+    <t>Map Layer Check</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Internet connection is OK 
+2. Standard Map Layer (default) is selected </t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open Open Street Map org
+2. Click on 'Layer' icon
+3. Select 'Tracestrack Topo'
 </t>
   </si>
   <si>
-    <t>Clean up all the input</t>
+    <t>1. OSM opened in browser
+2. Map Layer Option (Standard, CyclOSM, Cycle Map, Transport Map, Tracestrack Topo, Humanitarian, Shortbread, MapTiler OMT) has been displayed on the screen
+3. The map display change to Tracestrack Topo</t>
+  </si>
+  <si>
+    <t>Set the may layer back to 'Standard' , click 'closed' icon to close the Map Layers drawer</t>
   </si>
 </sst>
 </file>
@@ -99,7 +139,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -108,9 +148,6 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
@@ -398,11 +435,57 @@
       <c r="E2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="G2" s="3" t="s">
         <v>13</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>